<commit_message>
Checkpoint current experiment progress
</commit_message>
<xml_diff>
--- a/small test.xlsx
+++ b/small test.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Amy\002 救護車調度和損壞道路修復決策\005 程式\Taipei Case Test_(06-28)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1848FACE-3BAC-4695-B440-31CA8C09385C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AEFDF91-5829-45BD-9E9B-02007D302758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stress Test" sheetId="1" r:id="rId1"/>
-    <sheet name="Time Period" sheetId="3" r:id="rId2"/>
-    <sheet name="Sensitivity Analysis" sheetId="2" r:id="rId3"/>
-    <sheet name="README" sheetId="4" r:id="rId4"/>
+    <sheet name="fix ccp" sheetId="5" r:id="rId2"/>
+    <sheet name="Time Period" sheetId="3" r:id="rId3"/>
+    <sheet name="Sensitivity Analysis" sheetId="2" r:id="rId4"/>
+    <sheet name="README" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="167">
   <si>
     <t>test_id</t>
   </si>
@@ -90,9 +91,6 @@
   </si>
   <si>
     <t>ST25</t>
-  </si>
-  <si>
-    <t>Taipei 25%</t>
   </si>
   <si>
     <t>ST50</t>
@@ -534,10 +532,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>Taipei 10%</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>Taipei 50%</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -633,6 +627,125 @@
 CCP 15   -&gt; X: 1, Staff(V): 20, Amb(U):  9, MedicalSupply(Y): 860.00</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>全部抽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 25%</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>全部抽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 10%</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>CCP: 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>；</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>10%</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>CCP: 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>；20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>%</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>CCP: 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t>；30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>%</t>
+    </r>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -641,7 +754,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -774,6 +887,20 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="16">
@@ -1166,6 +1293,105 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="15" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="15" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="16" fillId="15" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1178,106 +1404,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="19" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="15" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="19" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="15" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="19" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="15" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="15" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="15" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1601,31 +1732,31 @@
     <col min="15" max="15" width="10" style="33" customWidth="1"/>
     <col min="16" max="16" width="11" style="33" customWidth="1"/>
     <col min="17" max="19" width="13" style="45" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="78"/>
+    <col min="20" max="16384" width="9" style="33"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
-        <v>139</v>
-      </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
-      <c r="R1" s="47"/>
-      <c r="S1" s="47"/>
+      <c r="A1" s="79" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="80"/>
+      <c r="S1" s="80"/>
     </row>
     <row r="2" spans="1:19" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="34" t="s">
@@ -1653,13 +1784,13 @@
         <v>7</v>
       </c>
       <c r="I2" s="34" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J2" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="K2" s="34" t="s">
         <v>140</v>
-      </c>
-      <c r="K2" s="34" t="s">
-        <v>141</v>
       </c>
       <c r="L2" s="34" t="s">
         <v>8</v>
@@ -1680,18 +1811,18 @@
         <v>13</v>
       </c>
       <c r="R2" s="35" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="S2" s="35" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="63.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>142</v>
+        <v>147</v>
+      </c>
+      <c r="B3" s="85" t="s">
+        <v>163</v>
       </c>
       <c r="C3" s="37">
         <v>23</v>
@@ -1712,7 +1843,7 @@
         <v>3386432.3</v>
       </c>
       <c r="I3" s="39" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J3" s="39">
         <v>3386432.3</v>
@@ -1749,8 +1880,8 @@
       <c r="A4" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="37" t="s">
-        <v>15</v>
+      <c r="B4" s="85" t="s">
+        <v>162</v>
       </c>
       <c r="C4" s="37">
         <v>58</v>
@@ -1771,7 +1902,7 @@
         <v>7428143.7599999998</v>
       </c>
       <c r="I4" s="39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J4" s="39">
         <v>7428143.7599999998</v>
@@ -1805,70 +1936,70 @@
       </c>
     </row>
     <row r="5" spans="1:19" ht="112.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="53" t="s">
-        <v>143</v>
-      </c>
-      <c r="C5" s="53">
+      <c r="A5" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="47">
         <v>115</v>
       </c>
-      <c r="D5" s="53">
+      <c r="D5" s="47">
         <v>8</v>
       </c>
-      <c r="E5" s="52">
+      <c r="E5" s="46">
         <v>10</v>
       </c>
-      <c r="F5" s="52">
+      <c r="F5" s="46">
         <v>20</v>
       </c>
-      <c r="G5" s="52">
+      <c r="G5" s="46">
         <v>8</v>
       </c>
-      <c r="H5" s="54">
+      <c r="H5" s="48">
         <v>18742679.710000001</v>
       </c>
-      <c r="I5" s="55" t="s">
+      <c r="I5" s="49" t="s">
+        <v>144</v>
+      </c>
+      <c r="J5" s="48">
+        <v>13436423.32</v>
+      </c>
+      <c r="K5" s="48">
+        <v>18742679.710000001</v>
+      </c>
+      <c r="L5" s="48" t="s">
+        <v>145</v>
+      </c>
+      <c r="M5" s="48">
+        <v>532744</v>
+      </c>
+      <c r="N5" s="48">
+        <v>235236</v>
+      </c>
+      <c r="O5" s="48">
+        <v>1</v>
+      </c>
+      <c r="P5" s="48">
+        <v>758574</v>
+      </c>
+      <c r="Q5" s="50">
+        <v>0.283111</v>
+      </c>
+      <c r="R5" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="J5" s="54">
-        <v>13436423.32</v>
-      </c>
-      <c r="K5" s="54">
-        <v>18742679.710000001</v>
-      </c>
-      <c r="L5" s="54" t="s">
-        <v>147</v>
-      </c>
-      <c r="M5" s="54">
-        <v>532744</v>
-      </c>
-      <c r="N5" s="54">
-        <v>235236</v>
-      </c>
-      <c r="O5" s="54">
-        <v>1</v>
-      </c>
-      <c r="P5" s="54">
-        <v>758574</v>
-      </c>
-      <c r="Q5" s="56">
-        <v>0.283111</v>
-      </c>
-      <c r="R5" s="56" t="s">
-        <v>148</v>
-      </c>
-      <c r="S5" s="56" t="s">
-        <v>148</v>
+      <c r="S5" s="50" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="43.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C6" s="37">
         <v>58</v>
@@ -1889,7 +2020,7 @@
         <v>7435282.1600000001</v>
       </c>
       <c r="I6" s="43" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J6" s="43">
         <v>7432592.3300000001</v>
@@ -1924,10 +2055,10 @@
     </row>
     <row r="7" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C7" s="37">
         <v>58</v>
@@ -1948,7 +2079,7 @@
         <v>7428143.7599999998</v>
       </c>
       <c r="I7" s="39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J7" s="39">
         <v>7428143.7599999998</v>
@@ -1983,10 +2114,10 @@
     </row>
     <row r="8" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C8" s="37">
         <v>58</v>
@@ -2007,7 +2138,7 @@
         <v>7420813.8799999999</v>
       </c>
       <c r="I8" s="39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J8" s="39">
         <v>7092457.5599999996</v>
@@ -2041,62 +2172,62 @@
       </c>
     </row>
     <row r="9" spans="1:19" ht="47.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="52" t="s">
-        <v>154</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>136</v>
-      </c>
-      <c r="C9" s="53">
+      <c r="A9" s="46" t="s">
+        <v>152</v>
+      </c>
+      <c r="B9" s="47" t="s">
+        <v>135</v>
+      </c>
+      <c r="C9" s="47">
         <v>58</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="47">
         <v>4</v>
       </c>
-      <c r="E9" s="52">
+      <c r="E9" s="46">
         <v>5</v>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="46">
         <v>50</v>
       </c>
-      <c r="G9" s="52">
+      <c r="G9" s="46">
         <v>8</v>
       </c>
-      <c r="H9" s="54">
+      <c r="H9" s="48">
         <v>8010855.6299999999</v>
       </c>
-      <c r="I9" s="55" t="s">
-        <v>152</v>
-      </c>
-      <c r="J9" s="54">
+      <c r="I9" s="49" t="s">
+        <v>150</v>
+      </c>
+      <c r="J9" s="48">
         <v>7067295.0300000003</v>
       </c>
-      <c r="K9" s="54">
+      <c r="K9" s="48">
         <v>8010855.6299999999</v>
       </c>
-      <c r="L9" s="54" t="s">
-        <v>147</v>
-      </c>
-      <c r="M9" s="54">
+      <c r="L9" s="48" t="s">
+        <v>145</v>
+      </c>
+      <c r="M9" s="48">
         <v>376832</v>
       </c>
-      <c r="N9" s="54">
+      <c r="N9" s="48">
         <v>195419</v>
       </c>
-      <c r="O9" s="54">
+      <c r="O9" s="48">
         <v>1</v>
       </c>
-      <c r="P9" s="54">
+      <c r="P9" s="48">
         <v>1339285</v>
       </c>
-      <c r="Q9" s="56">
+      <c r="Q9" s="50">
         <v>0.117785</v>
       </c>
-      <c r="R9" s="56" t="s">
-        <v>148</v>
-      </c>
-      <c r="S9" s="56" t="s">
-        <v>148</v>
+      <c r="R9" s="50" t="s">
+        <v>146</v>
+      </c>
+      <c r="S9" s="50" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2109,6 +2240,437 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0F49013-DEE7-40D2-B26F-F6A2814300E8}">
+  <dimension ref="A1:S14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="17.75" customWidth="1"/>
+    <col min="8" max="8" width="22.125" customWidth="1"/>
+    <col min="9" max="9" width="56.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="79" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
+      <c r="J1" s="80"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="80"/>
+      <c r="S1" s="80"/>
+    </row>
+    <row r="2" spans="1:19" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="J2" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="K2" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="L2" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="34" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="R2" s="35" t="s">
+        <v>153</v>
+      </c>
+      <c r="S2" s="35" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="B3" s="86"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="38"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="38"/>
+      <c r="M3" s="38"/>
+      <c r="N3" s="38"/>
+      <c r="O3" s="38"/>
+      <c r="P3" s="38"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="40"/>
+    </row>
+    <row r="4" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="36"/>
+      <c r="B4" s="86"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="39"/>
+      <c r="J4" s="39"/>
+      <c r="K4" s="39"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="38"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="38"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="40"/>
+      <c r="S4" s="40"/>
+    </row>
+    <row r="5" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="36"/>
+      <c r="B5" s="86"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="39"/>
+      <c r="J5" s="39"/>
+      <c r="K5" s="39"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="38"/>
+      <c r="Q5" s="40"/>
+      <c r="R5" s="40"/>
+      <c r="S5" s="40"/>
+    </row>
+    <row r="6" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="36"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="39"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="38"/>
+      <c r="P6" s="38"/>
+      <c r="Q6" s="40"/>
+      <c r="R6" s="40"/>
+      <c r="S6" s="40"/>
+    </row>
+    <row r="7" spans="1:19" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="36"/>
+      <c r="B7" s="86" t="s">
+        <v>164</v>
+      </c>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37">
+        <v>8</v>
+      </c>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36">
+        <v>5</v>
+      </c>
+      <c r="G7" s="36">
+        <v>8</v>
+      </c>
+      <c r="H7" s="38"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="38"/>
+      <c r="M7" s="38"/>
+      <c r="N7" s="38"/>
+      <c r="O7" s="38"/>
+      <c r="P7" s="38"/>
+      <c r="Q7" s="40"/>
+      <c r="R7" s="40"/>
+      <c r="S7" s="40"/>
+    </row>
+    <row r="8" spans="1:19" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="86" t="s">
+        <v>165</v>
+      </c>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37">
+        <v>8</v>
+      </c>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36">
+        <v>5</v>
+      </c>
+      <c r="G8" s="36">
+        <v>8</v>
+      </c>
+      <c r="H8" s="38"/>
+      <c r="I8" s="39"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="39"/>
+      <c r="L8" s="38"/>
+      <c r="M8" s="38"/>
+      <c r="N8" s="38"/>
+      <c r="O8" s="38"/>
+      <c r="P8" s="38"/>
+      <c r="Q8" s="40"/>
+      <c r="R8" s="40"/>
+      <c r="S8" s="40"/>
+    </row>
+    <row r="9" spans="1:19" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="36"/>
+      <c r="B9" s="86" t="s">
+        <v>166</v>
+      </c>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37">
+        <v>8</v>
+      </c>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36">
+        <v>5</v>
+      </c>
+      <c r="G9" s="36">
+        <v>8</v>
+      </c>
+      <c r="H9" s="38"/>
+      <c r="I9" s="39"/>
+      <c r="J9" s="39"/>
+      <c r="K9" s="39"/>
+      <c r="L9" s="38"/>
+      <c r="M9" s="38"/>
+      <c r="N9" s="38"/>
+      <c r="O9" s="38"/>
+      <c r="P9" s="38"/>
+      <c r="Q9" s="40"/>
+      <c r="R9" s="40"/>
+      <c r="S9" s="40"/>
+    </row>
+    <row r="10" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="46" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="47" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="47"/>
+      <c r="D10" s="37">
+        <v>8</v>
+      </c>
+      <c r="E10" s="46"/>
+      <c r="F10" s="36">
+        <v>5</v>
+      </c>
+      <c r="G10" s="46">
+        <v>8</v>
+      </c>
+      <c r="H10" s="48"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
+      <c r="M10" s="48"/>
+      <c r="N10" s="48"/>
+      <c r="O10" s="48"/>
+      <c r="P10" s="48"/>
+      <c r="Q10" s="50"/>
+      <c r="R10" s="50"/>
+      <c r="S10" s="50"/>
+    </row>
+    <row r="11" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="B11" s="42" t="s">
+        <v>133</v>
+      </c>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37">
+        <v>8</v>
+      </c>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36">
+        <v>5</v>
+      </c>
+      <c r="G11" s="41">
+        <v>8</v>
+      </c>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="44"/>
+      <c r="R11" s="44"/>
+      <c r="S11" s="44"/>
+    </row>
+    <row r="12" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="42" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37">
+        <v>8</v>
+      </c>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36">
+        <v>5</v>
+      </c>
+      <c r="G12" s="41">
+        <v>8</v>
+      </c>
+      <c r="H12" s="38"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="38"/>
+      <c r="P12" s="38"/>
+      <c r="Q12" s="40"/>
+      <c r="R12" s="40"/>
+      <c r="S12" s="40"/>
+    </row>
+    <row r="13" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A13" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37">
+        <v>8</v>
+      </c>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36">
+        <v>5</v>
+      </c>
+      <c r="G13" s="41">
+        <v>8</v>
+      </c>
+      <c r="H13" s="38"/>
+      <c r="I13" s="39"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="38"/>
+      <c r="P13" s="38"/>
+      <c r="Q13" s="40"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="40"/>
+    </row>
+    <row r="14" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="46" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="47" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="47"/>
+      <c r="D14" s="37">
+        <v>8</v>
+      </c>
+      <c r="E14" s="46"/>
+      <c r="F14" s="36">
+        <v>5</v>
+      </c>
+      <c r="G14" s="46">
+        <v>8</v>
+      </c>
+      <c r="H14" s="48"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="48"/>
+      <c r="N14" s="48"/>
+      <c r="O14" s="48"/>
+      <c r="P14" s="48"/>
+      <c r="Q14" s="50"/>
+      <c r="R14" s="50"/>
+      <c r="S14" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:S1"/>
+  </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
@@ -2124,279 +2686,279 @@
     <col min="9" max="9" width="13" style="7" customWidth="1"/>
     <col min="10" max="11" width="14" style="7" customWidth="1"/>
     <col min="12" max="12" width="10.25" style="7" customWidth="1"/>
-    <col min="13" max="13" width="16.25" style="83" customWidth="1"/>
-    <col min="14" max="14" width="16.875" style="86" customWidth="1"/>
-    <col min="15" max="16" width="10.75" style="86" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.25" style="72" customWidth="1"/>
+    <col min="14" max="14" width="16.875" style="75" customWidth="1"/>
+    <col min="15" max="16" width="10.75" style="75" bestFit="1" customWidth="1"/>
     <col min="17" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="76" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="78"/>
+    </row>
+    <row r="2" spans="1:16" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="69"/>
-    </row>
-    <row r="2" spans="1:16" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="57" t="s">
+      <c r="D2" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="51" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="51" t="s">
+        <v>136</v>
+      </c>
+      <c r="G2" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" s="51" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2" s="51" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="51" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="52" t="s">
+        <v>153</v>
+      </c>
+      <c r="P2" s="61" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="62" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="53">
+        <v>4</v>
+      </c>
+      <c r="D3" s="53" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="54">
+        <v>5599642.29</v>
+      </c>
+      <c r="F3" s="54" t="s">
+        <v>159</v>
+      </c>
+      <c r="G3" s="54">
+        <v>5599544</v>
+      </c>
+      <c r="H3" s="54">
+        <v>5599642.29</v>
+      </c>
+      <c r="I3" s="54">
+        <v>115.15</v>
+      </c>
+      <c r="J3" s="54">
+        <v>75392</v>
+      </c>
+      <c r="K3" s="54">
+        <v>39139</v>
+      </c>
+      <c r="L3" s="55">
         <v>1</v>
       </c>
-      <c r="C2" s="57" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="57" t="s">
+      <c r="M3" s="68">
+        <v>231184</v>
+      </c>
+      <c r="N3" s="69">
+        <v>1.8E-5</v>
+      </c>
+      <c r="O3" s="69">
+        <v>2.4441000000000001E-2</v>
+      </c>
+      <c r="P3" s="70">
+        <v>2.7699999999999999E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="62" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="53">
+        <v>8</v>
+      </c>
+      <c r="D4" s="53" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="56">
+        <v>7428143.7599999998</v>
+      </c>
+      <c r="F4" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="G2" s="57" t="s">
-        <v>140</v>
-      </c>
-      <c r="H2" s="57" t="s">
-        <v>141</v>
-      </c>
-      <c r="I2" s="57" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" s="57" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" s="57" t="s">
-        <v>10</v>
-      </c>
-      <c r="L2" s="57" t="s">
-        <v>11</v>
-      </c>
-      <c r="M2" s="57" t="s">
-        <v>12</v>
-      </c>
-      <c r="N2" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="O2" s="58" t="s">
-        <v>155</v>
-      </c>
-      <c r="P2" s="71" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" s="59" customFormat="1" ht="43.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="72" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="60" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="60">
-        <v>4</v>
-      </c>
-      <c r="D3" s="60" t="s">
+      <c r="G4" s="57">
+        <v>7428143.7599999998</v>
+      </c>
+      <c r="H4" s="57">
+        <v>7427963.7800000003</v>
+      </c>
+      <c r="I4" s="56">
+        <v>267.75</v>
+      </c>
+      <c r="J4" s="56">
+        <v>150752</v>
+      </c>
+      <c r="K4" s="56">
+        <v>78179</v>
+      </c>
+      <c r="L4" s="58">
+        <v>1</v>
+      </c>
+      <c r="M4" s="56">
+        <v>241578</v>
+      </c>
+      <c r="N4" s="59">
+        <v>2.4000000000000001E-5</v>
+      </c>
+      <c r="O4" s="59">
+        <v>6.0920000000000002E-2</v>
+      </c>
+      <c r="P4" s="63">
+        <v>3.9620000000000002E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="62" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="53">
+        <v>16</v>
+      </c>
+      <c r="D5" s="53" t="s">
         <v>157</v>
       </c>
-      <c r="E3" s="61">
-        <v>5599642.29</v>
-      </c>
-      <c r="F3" s="61" t="s">
+      <c r="E5" s="54">
+        <v>13975899.300000001</v>
+      </c>
+      <c r="F5" s="54" t="s">
+        <v>160</v>
+      </c>
+      <c r="G5" s="54">
+        <v>13946011.689999999</v>
+      </c>
+      <c r="H5" s="54">
+        <v>13975899.300000001</v>
+      </c>
+      <c r="I5" s="54">
+        <v>570.09</v>
+      </c>
+      <c r="J5" s="54">
+        <v>301472</v>
+      </c>
+      <c r="K5" s="54">
+        <v>156259</v>
+      </c>
+      <c r="L5" s="55">
+        <v>1</v>
+      </c>
+      <c r="M5" s="68">
+        <v>188208</v>
+      </c>
+      <c r="N5" s="69">
+        <v>2.1389999999999998E-3</v>
+      </c>
+      <c r="O5" s="69">
+        <v>7.5605000000000006E-2</v>
+      </c>
+      <c r="P5" s="70">
+        <v>7.4520000000000003E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="79.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="64" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="65" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="65">
+        <v>32</v>
+      </c>
+      <c r="D6" s="65" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="66">
+        <v>166722852.47999999</v>
+      </c>
+      <c r="F6" s="66" t="s">
         <v>161</v>
       </c>
-      <c r="G3" s="61">
-        <v>5599544</v>
-      </c>
-      <c r="H3" s="61">
-        <v>5599642.29</v>
-      </c>
-      <c r="I3" s="61">
-        <v>115.15</v>
-      </c>
-      <c r="J3" s="61">
-        <v>75392</v>
-      </c>
-      <c r="K3" s="61">
-        <v>39139</v>
-      </c>
-      <c r="L3" s="62">
+      <c r="G6" s="66">
+        <v>166676212.56</v>
+      </c>
+      <c r="H6" s="66">
+        <v>166722852.47999999</v>
+      </c>
+      <c r="I6" s="66">
+        <v>29.66</v>
+      </c>
+      <c r="J6" s="66">
+        <v>602912</v>
+      </c>
+      <c r="K6" s="66">
+        <v>312419</v>
+      </c>
+      <c r="L6" s="67">
         <v>1</v>
       </c>
-      <c r="M3" s="79">
-        <v>231184</v>
-      </c>
-      <c r="N3" s="80">
-        <v>1.8E-5</v>
-      </c>
-      <c r="O3" s="80">
-        <v>2.4441000000000001E-2</v>
-      </c>
-      <c r="P3" s="81">
-        <v>2.7699999999999999E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" s="59" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="72" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="60" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="60">
-        <v>8</v>
-      </c>
-      <c r="D4" s="60" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" s="63">
-        <v>7428143.7599999998</v>
-      </c>
-      <c r="F4" s="64" t="s">
-        <v>138</v>
-      </c>
-      <c r="G4" s="64">
-        <v>7428143.7599999998</v>
-      </c>
-      <c r="H4" s="64">
-        <v>7427963.7800000003</v>
-      </c>
-      <c r="I4" s="63">
-        <v>267.75</v>
-      </c>
-      <c r="J4" s="63">
-        <v>150752</v>
-      </c>
-      <c r="K4" s="63">
-        <v>78179</v>
-      </c>
-      <c r="L4" s="65">
-        <v>1</v>
-      </c>
-      <c r="M4" s="63">
-        <v>241578</v>
-      </c>
-      <c r="N4" s="66">
-        <v>2.4000000000000001E-5</v>
-      </c>
-      <c r="O4" s="66">
-        <v>6.0920000000000002E-2</v>
-      </c>
-      <c r="P4" s="73">
-        <v>3.9620000000000002E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" s="59" customFormat="1" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="72" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="60">
-        <v>16</v>
-      </c>
-      <c r="D5" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="E5" s="61">
-        <v>13975899.300000001</v>
-      </c>
-      <c r="F5" s="61" t="s">
-        <v>162</v>
-      </c>
-      <c r="G5" s="61">
-        <v>13946011.689999999</v>
-      </c>
-      <c r="H5" s="61">
-        <v>13975899.300000001</v>
-      </c>
-      <c r="I5" s="61">
-        <v>570.09</v>
-      </c>
-      <c r="J5" s="61">
-        <v>301472</v>
-      </c>
-      <c r="K5" s="61">
-        <v>156259</v>
-      </c>
-      <c r="L5" s="62">
-        <v>1</v>
-      </c>
-      <c r="M5" s="79">
-        <v>188208</v>
-      </c>
-      <c r="N5" s="80">
-        <v>2.1389999999999998E-3</v>
-      </c>
-      <c r="O5" s="80">
-        <v>7.5605000000000006E-2</v>
-      </c>
-      <c r="P5" s="81">
-        <v>7.4520000000000003E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" s="59" customFormat="1" ht="79.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="74" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="75" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="75">
-        <v>32</v>
-      </c>
-      <c r="D6" s="75" t="s">
-        <v>160</v>
-      </c>
-      <c r="E6" s="76">
-        <v>166722852.47999999</v>
-      </c>
-      <c r="F6" s="76" t="s">
-        <v>163</v>
-      </c>
-      <c r="G6" s="76">
-        <v>166676212.56</v>
-      </c>
-      <c r="H6" s="76">
-        <v>166722852.47999999</v>
-      </c>
-      <c r="I6" s="76">
-        <v>29.66</v>
-      </c>
-      <c r="J6" s="76">
-        <v>602912</v>
-      </c>
-      <c r="K6" s="76">
-        <v>312419</v>
-      </c>
-      <c r="L6" s="77">
-        <v>1</v>
-      </c>
-      <c r="M6" s="82">
+      <c r="M6" s="71">
         <v>9602</v>
       </c>
-      <c r="N6" s="84">
+      <c r="N6" s="73">
         <v>2.7999999999999998E-4</v>
       </c>
-      <c r="O6" s="84">
+      <c r="O6" s="73">
         <v>5.9599999999999996E-4</v>
       </c>
-      <c r="P6" s="85">
+      <c r="P6" s="74">
         <v>3.3500000000000001E-4</v>
       </c>
     </row>
@@ -2409,7 +2971,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
@@ -2430,31 +2992,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="48" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="49"/>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="49"/>
-      <c r="U1" s="49"/>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
+      <c r="A1" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="82"/>
+      <c r="E1" s="82"/>
+      <c r="F1" s="82"/>
+      <c r="G1" s="82"/>
+      <c r="H1" s="82"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="82"/>
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+      <c r="S1" s="82"/>
+      <c r="T1" s="82"/>
+      <c r="U1" s="82"/>
+      <c r="V1" s="82"/>
+      <c r="W1" s="82"/>
     </row>
     <row r="2" spans="1:23" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
@@ -2464,19 +3026,19 @@
         <v>1</v>
       </c>
       <c r="C2" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>20</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>21</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>22</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>8</v>
@@ -2485,60 +3047,60 @@
         <v>13</v>
       </c>
       <c r="J2" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="K2" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>128</v>
-      </c>
       <c r="M2" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="N2" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="O2" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="O2" s="11" t="s">
+      <c r="P2" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="Q2" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="R2" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="S2" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="T2" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="U2" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="U2" s="11" t="s">
-        <v>126</v>
-      </c>
       <c r="V2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="W2" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="W2" s="9" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>26</v>
-      </c>
       <c r="C3" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>130</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>131</v>
       </c>
       <c r="E3" s="14"/>
       <c r="F3" s="14"/>
@@ -2559,21 +3121,21 @@
       <c r="U3" s="14"/>
       <c r="V3" s="14"/>
       <c r="W3" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="C4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>31</v>
-      </c>
       <c r="D4" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E4" s="17"/>
       <c r="F4" s="17"/>
@@ -2597,16 +3159,16 @@
     </row>
     <row r="5" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>33</v>
-      </c>
       <c r="D5" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E5" s="17"/>
       <c r="F5" s="17"/>
@@ -2630,16 +3192,16 @@
     </row>
     <row r="6" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>35</v>
-      </c>
       <c r="D6" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
@@ -2663,16 +3225,16 @@
     </row>
     <row r="7" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="C7" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>38</v>
-      </c>
       <c r="D7" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E7" s="20"/>
       <c r="F7" s="20"/>
@@ -2696,16 +3258,16 @@
     </row>
     <row r="8" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>40</v>
-      </c>
       <c r="D8" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="20"/>
       <c r="F8" s="20"/>
@@ -2729,16 +3291,16 @@
     </row>
     <row r="9" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>42</v>
-      </c>
       <c r="D9" s="19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E9" s="20"/>
       <c r="F9" s="20"/>
@@ -2762,16 +3324,16 @@
     </row>
     <row r="10" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="C10" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="22" t="s">
-        <v>45</v>
-      </c>
       <c r="D10" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="23"/>
       <c r="F10" s="23"/>
@@ -2795,16 +3357,16 @@
     </row>
     <row r="11" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="22" t="s">
-        <v>47</v>
-      </c>
       <c r="D11" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E11" s="23"/>
       <c r="F11" s="23"/>
@@ -2828,16 +3390,16 @@
     </row>
     <row r="12" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>49</v>
-      </c>
       <c r="D12" s="22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -2861,16 +3423,16 @@
     </row>
     <row r="13" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="C13" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="25" t="s">
-        <v>52</v>
-      </c>
       <c r="D13" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="26"/>
       <c r="F13" s="26"/>
@@ -2894,16 +3456,16 @@
     </row>
     <row r="14" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="25" t="s">
-        <v>54</v>
-      </c>
       <c r="D14" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="26"/>
       <c r="F14" s="26"/>
@@ -2927,16 +3489,16 @@
     </row>
     <row r="15" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>56</v>
-      </c>
       <c r="D15" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" s="26"/>
       <c r="F15" s="26"/>
@@ -2960,16 +3522,16 @@
     </row>
     <row r="16" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="C16" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="28" t="s">
+      <c r="D16" s="28" t="s">
         <v>59</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>60</v>
       </c>
       <c r="E16" s="29"/>
       <c r="F16" s="29"/>
@@ -2990,21 +3552,21 @@
       <c r="U16" s="29"/>
       <c r="V16" s="29"/>
       <c r="W16" s="28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="C17" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="D17" s="31" t="s">
         <v>64</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>65</v>
       </c>
       <c r="E17" s="32"/>
       <c r="F17" s="32"/>
@@ -3025,7 +3587,7 @@
       <c r="U17" s="32"/>
       <c r="V17" s="32"/>
       <c r="W17" s="31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3037,7 +3599,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
@@ -3047,33 +3609,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="50" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" s="51"/>
+      <c r="A1" s="83" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="84"/>
     </row>
     <row r="2" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3082,32 +3644,32 @@
     </row>
     <row r="6" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B6" s="5"/>
     </row>
     <row r="7" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3116,64 +3678,64 @@
     </row>
     <row r="11" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B11" s="5"/>
     </row>
     <row r="12" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -3182,56 +3744,56 @@
     </row>
     <row r="20" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B20" s="5"/>
     </row>
     <row r="21" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
B&BC + Warm Start + folder organization
</commit_message>
<xml_diff>
--- a/small test.xlsx
+++ b/small test.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Amy\002 救護車調度和損壞道路修復決策\005 程式\Taipei Case Test_(06-28)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FA11F8-F4DD-405B-8952-0A13D6E5D92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE66A29-76AF-4E66-ADFC-59D7C501E5E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="111">
   <si>
     <t>test_id</t>
   </si>
@@ -481,6 +481,14 @@
   </si>
   <si>
     <t>Time Period x16</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>VSS(%)</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>EVPI(%)</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -1783,10 +1791,10 @@
         <v>13</v>
       </c>
       <c r="Q17" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="R17" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>